<commit_message>
more plot for detectability
</commit_message>
<xml_diff>
--- a/cosine-similarity/essay_similarity_results.xlsx
+++ b/cosine-similarity/essay_similarity_results.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Groupby_Length_Humanizer" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Groupby_Humanizer" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9041,4 +9043,555 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>humanizer</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>TF-IDF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>SBERT</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Nemotron</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AIHumanizer</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.7478047423131782</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.8797962486743927</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.960100245475769</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Grammarly</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.6792858532162303</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8390336930751801</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9259900152683258</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HumanizeAI</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.7377228977399604</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.8713624835014343</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9416908383369446</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Quillbot</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.7445938695027987</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.913640683889389</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9613904893398285</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>UndetectableAI</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.6594376472561455</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.8300792396068573</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.9095285296440124</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>writehuman.ai</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.7125493103838961</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.8723353505134582</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.9126749098300934</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AIHumanizer</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.67124129629361</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.8828529059886933</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.9547171771526337</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Grammarly</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.6451254325665119</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.8514619588851928</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.9374411225318908</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HumanizeAI</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.6473583156716725</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.8776766896247864</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.9194575548171997</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Quillbot</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.6745243310147881</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.9204445719718933</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.9571266531944275</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>UndetectableAI</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.585155636918684</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.8417653203010559</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.8917437553405761</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>writehuman.ai</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.6534776274697405</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.8560736378033956</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.883232957786984</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>AIHumanizer</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.5673665458177093</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.8777785360813141</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.9446422159671783</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Grammarly</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.649253268558232</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.8732444643974304</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.9419403731822967</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HumanizeAI</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.5594946544345951</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.867990231513977</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.9207612216472626</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Quillbot</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.5923681611263996</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.9033341825008392</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.9466703176498413</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>UndetectableAI</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.536926623791583</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.8466940283775329</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.887037044763565</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>writehuman.ai</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.5690659149569661</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.8508399844169616</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.8855505645275116</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>humanizer</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>TF-IDF</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>SBERT</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Nemotron</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AIHumanizer</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.6621375281414992</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.8801425635814667</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.9531532128651937</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Grammarly</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.6578881847803246</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.8545800387859345</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.9351238369941711</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HumanizeAI</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.6481919559487427</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.8723431348800659</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.9273032049338022</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Quillbot</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.6704954538813287</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.9124731461207072</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.9550624867280324</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>UndetectableAI</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.5938399693221376</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.8395128627618154</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.8961031099160512</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>writehuman.ai</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.6447396862288375</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.859876416880509</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.8941845297813416</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>